<commit_message>
broke/fix coinc trig adding mask, update constraint, alleviate the fifo transfer async thing
</commit_message>
<xml_diff>
--- a/doc/flower-register-map.xlsx
+++ b/doc/flower-register-map.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\clean\FLOWER-BOARD-Firmware\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\dev\FLOWER-board-firmware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B20BF66-5D7C-4842-8203-FA81531C5763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69701C28-00A0-4286-996E-2D1F345790AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registers" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="247">
   <si>
     <t>Register Map</t>
   </si>
@@ -684,27 +684,6 @@
     <t>Beam 8 Trigger</t>
   </si>
   <si>
-    <t>Beam 9 Trigger</t>
-  </si>
-  <si>
-    <t>Beam 10 Trigger</t>
-  </si>
-  <si>
-    <t>Beam 11 Trigger</t>
-  </si>
-  <si>
-    <t>Beam 12 Trigger</t>
-  </si>
-  <si>
-    <t>Beam 13 Trigger</t>
-  </si>
-  <si>
-    <t>Beam 14 Trigger</t>
-  </si>
-  <si>
-    <t>Beam 15 Trigger</t>
-  </si>
-  <si>
     <t>Phased Trigger</t>
   </si>
   <si>
@@ -721,27 +700,6 @@
   </si>
   <si>
     <t>Phased Servo</t>
-  </si>
-  <si>
-    <t>Beam 15 Servo</t>
-  </si>
-  <si>
-    <t>Beam 14 Servo</t>
-  </si>
-  <si>
-    <t>Beam 13 Servo</t>
-  </si>
-  <si>
-    <t>Beam 12 Servo</t>
-  </si>
-  <si>
-    <t>Beam 11 Servo</t>
-  </si>
-  <si>
-    <t>Beam 10 Servo</t>
-  </si>
-  <si>
-    <t>Beam 9 Servo</t>
   </si>
   <si>
     <t>Beam 8 Servo</t>
@@ -1799,7 +1757,7 @@
         <v>182</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
       <c r="E24" t="s">
         <v>6</v>
@@ -1819,7 +1777,7 @@
         <v>183</v>
       </c>
       <c r="D25" s="40" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="E25" t="s">
         <v>6</v>
@@ -2137,7 +2095,7 @@
         <v>40</v>
       </c>
       <c r="D48" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="E48" t="s">
         <v>6</v>
@@ -2775,10 +2733,10 @@
         <v>x50</v>
       </c>
       <c r="C87" s="42" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="D87" s="43" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="E87" s="42" t="s">
         <v>48</v>
@@ -2797,16 +2755,16 @@
         <v>x51</v>
       </c>
       <c r="C88" s="42" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="D88" s="43" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="E88" s="42" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="F88" s="43" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
@@ -2991,7 +2949,7 @@
         <v>x5B</v>
       </c>
       <c r="C98" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>155</v>
@@ -3610,13 +3568,13 @@
         <v>x80</v>
       </c>
       <c r="C135" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D135" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E135" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
@@ -3629,13 +3587,13 @@
         <v>x81</v>
       </c>
       <c r="C136" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D136" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E136" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
@@ -3648,13 +3606,13 @@
         <v>x82</v>
       </c>
       <c r="C137" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D137" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E137" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
@@ -3667,13 +3625,13 @@
         <v>x83</v>
       </c>
       <c r="C138" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D138" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E138" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
@@ -3686,13 +3644,13 @@
         <v>x84</v>
       </c>
       <c r="C139" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D139" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E139" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
@@ -3705,13 +3663,13 @@
         <v>x85</v>
       </c>
       <c r="C140" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D140" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E140" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
@@ -3724,13 +3682,13 @@
         <v>x86</v>
       </c>
       <c r="C141" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D141" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E141" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
@@ -3743,13 +3701,13 @@
         <v>x87</v>
       </c>
       <c r="C142" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D142" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E142" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
@@ -3762,13 +3720,13 @@
         <v>x88</v>
       </c>
       <c r="C143" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D143" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E143" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
@@ -3781,13 +3739,13 @@
         <v>x89</v>
       </c>
       <c r="C144" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D144" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E144" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
@@ -3800,13 +3758,13 @@
         <v>x8A</v>
       </c>
       <c r="C145" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D145" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E145" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
@@ -3819,13 +3777,13 @@
         <v>x8B</v>
       </c>
       <c r="C146" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D146" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E146" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
@@ -3838,13 +3796,13 @@
         <v>x8C</v>
       </c>
       <c r="C147" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D147" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E147" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
@@ -3857,13 +3815,13 @@
         <v>x8D</v>
       </c>
       <c r="C148" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D148" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E148" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
@@ -3876,13 +3834,13 @@
         <v>x8E</v>
       </c>
       <c r="C149" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D149" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E149" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
@@ -3895,13 +3853,13 @@
         <v>x8F</v>
       </c>
       <c r="C150" s="40" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D150" s="40" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E150" s="40" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
@@ -5038,7 +4996,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91517B1F-406D-4F65-BBD5-9E59DD7F84C2}">
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" customWidth="1"/>
@@ -5052,16 +5010,16 @@
         <v>201</v>
       </c>
       <c r="B1" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="C1" t="s">
         <v>202</v>
       </c>
       <c r="D1" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="F1" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -5072,7 +5030,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -5098,7 +5056,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -5111,7 +5069,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -5124,7 +5082,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -5137,7 +5095,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -5630,7 +5588,7 @@
         <v>18</v>
       </c>
       <c r="C38" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="D38" t="s">
         <v>190</v>
@@ -5790,7 +5748,7 @@
         <v>23</v>
       </c>
       <c r="C48" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D48" t="s">
         <v>190</v>
@@ -5870,7 +5828,7 @@
         <v>25</v>
       </c>
       <c r="C53" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D53" t="s">
         <v>190</v>
@@ -5886,7 +5844,7 @@
         <v>26</v>
       </c>
       <c r="C54" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D54" t="s">
         <v>190</v>
@@ -5902,7 +5860,7 @@
         <v>26</v>
       </c>
       <c r="C55" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D55" t="s">
         <v>190</v>
@@ -5918,7 +5876,7 @@
         <v>27</v>
       </c>
       <c r="C56" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D56" t="s">
         <v>190</v>
@@ -5934,7 +5892,7 @@
         <v>27</v>
       </c>
       <c r="C57" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D57" t="s">
         <v>190</v>
@@ -5950,10 +5908,10 @@
         <v>28</v>
       </c>
       <c r="C58" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="D58" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
@@ -5966,10 +5924,10 @@
         <v>28</v>
       </c>
       <c r="C59" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="D59" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
@@ -5982,10 +5940,10 @@
         <v>29</v>
       </c>
       <c r="C60" t="s">
-        <v>239</v>
+        <v>207</v>
       </c>
       <c r="D60" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
@@ -5998,10 +5956,10 @@
         <v>29</v>
       </c>
       <c r="C61" t="s">
-        <v>238</v>
+        <v>208</v>
       </c>
       <c r="D61" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
@@ -6014,10 +5972,10 @@
         <v>30</v>
       </c>
       <c r="C62" t="s">
-        <v>237</v>
+        <v>209</v>
       </c>
       <c r="D62" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
@@ -6030,10 +5988,10 @@
         <v>30</v>
       </c>
       <c r="C63" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="D63" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
@@ -6046,10 +6004,10 @@
         <v>31</v>
       </c>
       <c r="C64" t="s">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="D64" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
@@ -6062,10 +6020,10 @@
         <v>31</v>
       </c>
       <c r="C65" t="s">
-        <v>234</v>
+        <v>212</v>
       </c>
       <c r="D65" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
@@ -6078,10 +6036,10 @@
         <v>32</v>
       </c>
       <c r="C66" t="s">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="D66" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
@@ -6094,10 +6052,10 @@
         <v>32</v>
       </c>
       <c r="C67" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="D67" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
@@ -6110,10 +6068,10 @@
         <v>33</v>
       </c>
       <c r="C68" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="D68" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
@@ -6126,10 +6084,10 @@
         <v>33</v>
       </c>
       <c r="C69" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="D69" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
@@ -6142,10 +6100,10 @@
         <v>34</v>
       </c>
       <c r="C70" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="D70" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
@@ -6158,10 +6116,10 @@
         <v>34</v>
       </c>
       <c r="C71" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="D71" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
@@ -6174,7 +6132,7 @@
         <v>35</v>
       </c>
       <c r="C72" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D72" t="s">
         <v>203</v>
@@ -6190,7 +6148,7 @@
         <v>35</v>
       </c>
       <c r="C73" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="D73" t="s">
         <v>203</v>
@@ -6206,7 +6164,7 @@
         <v>36</v>
       </c>
       <c r="C74" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="D74" t="s">
         <v>203</v>
@@ -6222,7 +6180,7 @@
         <v>36</v>
       </c>
       <c r="C75" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="D75" t="s">
         <v>203</v>
@@ -6238,7 +6196,7 @@
         <v>37</v>
       </c>
       <c r="C76" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="D76" t="s">
         <v>203</v>
@@ -6254,7 +6212,7 @@
         <v>37</v>
       </c>
       <c r="C77" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="D77" t="s">
         <v>203</v>
@@ -6270,10 +6228,10 @@
         <v>38</v>
       </c>
       <c r="C78" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D78" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
@@ -6286,10 +6244,10 @@
         <v>38</v>
       </c>
       <c r="C79" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="D79" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
@@ -6302,10 +6260,10 @@
         <v>39</v>
       </c>
       <c r="C80" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D80" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
@@ -6318,10 +6276,10 @@
         <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D81" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
@@ -6334,10 +6292,10 @@
         <v>40</v>
       </c>
       <c r="C82" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D82" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
@@ -6350,10 +6308,10 @@
         <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="D83" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
@@ -6366,10 +6324,10 @@
         <v>41</v>
       </c>
       <c r="C84" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D84" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
@@ -6382,10 +6340,10 @@
         <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D85" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
@@ -6398,10 +6356,10 @@
         <v>42</v>
       </c>
       <c r="C86" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="D86" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
@@ -6414,10 +6372,10 @@
         <v>42</v>
       </c>
       <c r="C87" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D87" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
@@ -6430,10 +6388,10 @@
         <v>43</v>
       </c>
       <c r="C88" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D88" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
@@ -6446,10 +6404,10 @@
         <v>43</v>
       </c>
       <c r="C89" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="D89" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
@@ -6462,10 +6420,10 @@
         <v>44</v>
       </c>
       <c r="C90" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D90" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
@@ -6478,10 +6436,10 @@
         <v>44</v>
       </c>
       <c r="C91" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="D91" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
@@ -6494,10 +6452,10 @@
         <v>45</v>
       </c>
       <c r="C92" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="D92" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
@@ -6510,10 +6468,10 @@
         <v>45</v>
       </c>
       <c r="C93" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D93" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
@@ -6526,10 +6484,10 @@
         <v>46</v>
       </c>
       <c r="C94" t="s">
-        <v>239</v>
+        <v>224</v>
       </c>
       <c r="D94" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
@@ -6542,10 +6500,10 @@
         <v>46</v>
       </c>
       <c r="C95" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="D95" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
@@ -6558,10 +6516,10 @@
         <v>47</v>
       </c>
       <c r="C96" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="D96" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
@@ -6574,681 +6532,9 @@
         <v>47</v>
       </c>
       <c r="C97" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="D97" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98">
-        <f t="shared" si="61"/>
-        <v>96</v>
-      </c>
-      <c r="B98">
-        <f t="shared" ref="B98" si="90">B96+1</f>
-        <v>48</v>
-      </c>
-      <c r="C98" t="s">
-        <v>235</v>
-      </c>
-      <c r="D98" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99">
-        <f t="shared" si="61"/>
-        <v>97</v>
-      </c>
-      <c r="B99">
-        <f t="shared" ref="B99" si="91">B98</f>
-        <v>48</v>
-      </c>
-      <c r="C99" t="s">
-        <v>234</v>
-      </c>
-      <c r="D99" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100">
-        <f t="shared" si="61"/>
-        <v>98</v>
-      </c>
-      <c r="B100">
-        <f t="shared" ref="B100" si="92">B98+1</f>
-        <v>49</v>
-      </c>
-      <c r="C100" t="s">
-        <v>233</v>
-      </c>
-      <c r="D100" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101">
-        <f t="shared" si="61"/>
-        <v>99</v>
-      </c>
-      <c r="B101">
-        <f t="shared" ref="B101" si="93">B100</f>
-        <v>49</v>
-      </c>
-      <c r="C101" t="s">
-        <v>232</v>
-      </c>
-      <c r="D101" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102">
-        <f t="shared" si="61"/>
-        <v>100</v>
-      </c>
-      <c r="B102">
-        <f t="shared" ref="B102" si="94">B100+1</f>
-        <v>50</v>
-      </c>
-      <c r="C102" t="s">
-        <v>231</v>
-      </c>
-      <c r="D102" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103">
-        <f t="shared" si="61"/>
-        <v>101</v>
-      </c>
-      <c r="B103">
-        <f t="shared" ref="B103" si="95">B102</f>
-        <v>50</v>
-      </c>
-      <c r="C103" t="s">
-        <v>230</v>
-      </c>
-      <c r="D103" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104">
-        <f t="shared" si="61"/>
-        <v>102</v>
-      </c>
-      <c r="B104">
-        <f t="shared" ref="B104" si="96">B102+1</f>
-        <v>51</v>
-      </c>
-      <c r="C104" t="s">
-        <v>229</v>
-      </c>
-      <c r="D104" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A105">
-        <f t="shared" si="61"/>
-        <v>103</v>
-      </c>
-      <c r="B105">
-        <f t="shared" ref="B105" si="97">B104</f>
-        <v>51</v>
-      </c>
-      <c r="C105" t="s">
-        <v>228</v>
-      </c>
-      <c r="D105" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A106">
-        <f t="shared" si="61"/>
-        <v>104</v>
-      </c>
-      <c r="B106">
-        <f t="shared" ref="B106" si="98">B104+1</f>
-        <v>52</v>
-      </c>
-      <c r="C106" t="s">
-        <v>222</v>
-      </c>
-      <c r="D106" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107">
-        <f t="shared" si="61"/>
-        <v>105</v>
-      </c>
-      <c r="B107">
-        <f t="shared" ref="B107" si="99">B106</f>
-        <v>52</v>
-      </c>
-      <c r="C107" t="s">
-        <v>206</v>
-      </c>
-      <c r="D107" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108">
-        <f t="shared" si="61"/>
-        <v>106</v>
-      </c>
-      <c r="B108">
-        <f t="shared" ref="B108" si="100">B106+1</f>
-        <v>53</v>
-      </c>
-      <c r="C108" t="s">
-        <v>207</v>
-      </c>
-      <c r="D108" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A109">
-        <f t="shared" si="61"/>
-        <v>107</v>
-      </c>
-      <c r="B109">
-        <f t="shared" ref="B109" si="101">B108</f>
-        <v>53</v>
-      </c>
-      <c r="C109" t="s">
-        <v>208</v>
-      </c>
-      <c r="D109" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A110">
-        <f t="shared" si="61"/>
-        <v>108</v>
-      </c>
-      <c r="B110">
-        <f t="shared" ref="B110" si="102">B108+1</f>
-        <v>54</v>
-      </c>
-      <c r="C110" t="s">
-        <v>209</v>
-      </c>
-      <c r="D110" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A111">
-        <f t="shared" si="61"/>
-        <v>109</v>
-      </c>
-      <c r="B111">
-        <f t="shared" ref="B111" si="103">B110</f>
-        <v>54</v>
-      </c>
-      <c r="C111" t="s">
-        <v>210</v>
-      </c>
-      <c r="D111" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A112">
-        <f t="shared" si="61"/>
-        <v>110</v>
-      </c>
-      <c r="B112">
-        <f t="shared" ref="B112" si="104">B110+1</f>
-        <v>55</v>
-      </c>
-      <c r="C112" t="s">
-        <v>211</v>
-      </c>
-      <c r="D112" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A113">
-        <f t="shared" si="61"/>
-        <v>111</v>
-      </c>
-      <c r="B113">
-        <f t="shared" ref="B113" si="105">B112</f>
-        <v>55</v>
-      </c>
-      <c r="C113" t="s">
-        <v>212</v>
-      </c>
-      <c r="D113" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A114">
-        <f t="shared" si="61"/>
-        <v>112</v>
-      </c>
-      <c r="B114">
-        <f t="shared" ref="B114" si="106">B112+1</f>
-        <v>56</v>
-      </c>
-      <c r="C114" t="s">
-        <v>213</v>
-      </c>
-      <c r="D114" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A115">
-        <f t="shared" si="61"/>
-        <v>113</v>
-      </c>
-      <c r="B115">
-        <f t="shared" ref="B115" si="107">B114</f>
-        <v>56</v>
-      </c>
-      <c r="C115" t="s">
-        <v>214</v>
-      </c>
-      <c r="D115" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A116">
-        <f t="shared" si="61"/>
-        <v>114</v>
-      </c>
-      <c r="B116">
-        <f t="shared" ref="B116" si="108">B114+1</f>
-        <v>57</v>
-      </c>
-      <c r="C116" t="s">
-        <v>215</v>
-      </c>
-      <c r="D116" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A117">
-        <f t="shared" si="61"/>
-        <v>115</v>
-      </c>
-      <c r="B117">
-        <f t="shared" ref="B117" si="109">B116</f>
-        <v>57</v>
-      </c>
-      <c r="C117" t="s">
-        <v>216</v>
-      </c>
-      <c r="D117" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A118">
-        <f t="shared" si="61"/>
-        <v>116</v>
-      </c>
-      <c r="B118">
-        <f t="shared" ref="B118" si="110">B116+1</f>
-        <v>58</v>
-      </c>
-      <c r="C118" t="s">
-        <v>217</v>
-      </c>
-      <c r="D118" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A119">
-        <f t="shared" si="61"/>
-        <v>117</v>
-      </c>
-      <c r="B119">
-        <f t="shared" ref="B119" si="111">B118</f>
-        <v>58</v>
-      </c>
-      <c r="C119" t="s">
-        <v>218</v>
-      </c>
-      <c r="D119" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A120">
-        <f t="shared" si="61"/>
-        <v>118</v>
-      </c>
-      <c r="B120">
-        <f t="shared" ref="B120" si="112">B118+1</f>
-        <v>59</v>
-      </c>
-      <c r="C120" t="s">
-        <v>219</v>
-      </c>
-      <c r="D120" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A121">
-        <f t="shared" si="61"/>
-        <v>119</v>
-      </c>
-      <c r="B121">
-        <f t="shared" ref="B121" si="113">B120</f>
-        <v>59</v>
-      </c>
-      <c r="C121" t="s">
-        <v>220</v>
-      </c>
-      <c r="D121" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A122">
-        <f t="shared" si="61"/>
-        <v>120</v>
-      </c>
-      <c r="B122">
-        <f t="shared" ref="B122" si="114">B120+1</f>
-        <v>60</v>
-      </c>
-      <c r="C122" t="s">
-        <v>221</v>
-      </c>
-      <c r="D122" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A123">
-        <f t="shared" si="61"/>
-        <v>121</v>
-      </c>
-      <c r="B123">
-        <f t="shared" ref="B123" si="115">B122</f>
-        <v>60</v>
-      </c>
-      <c r="C123" t="s">
-        <v>227</v>
-      </c>
-      <c r="D123" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A124">
-        <f t="shared" si="61"/>
-        <v>122</v>
-      </c>
-      <c r="B124">
-        <f t="shared" ref="B124" si="116">B122+1</f>
-        <v>61</v>
-      </c>
-      <c r="C124" t="s">
-        <v>223</v>
-      </c>
-      <c r="D124" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A125">
-        <f t="shared" si="61"/>
-        <v>123</v>
-      </c>
-      <c r="B125">
-        <f t="shared" ref="B125" si="117">B124</f>
-        <v>61</v>
-      </c>
-      <c r="C125" t="s">
-        <v>224</v>
-      </c>
-      <c r="D125" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A126">
-        <f t="shared" si="61"/>
-        <v>124</v>
-      </c>
-      <c r="B126">
-        <f t="shared" ref="B126" si="118">B124+1</f>
-        <v>62</v>
-      </c>
-      <c r="C126" t="s">
-        <v>225</v>
-      </c>
-      <c r="D126" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A127">
-        <f t="shared" si="61"/>
-        <v>125</v>
-      </c>
-      <c r="B127">
-        <f t="shared" ref="B127" si="119">B126</f>
-        <v>62</v>
-      </c>
-      <c r="C127" t="s">
-        <v>226</v>
-      </c>
-      <c r="D127" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A128">
-        <f t="shared" si="61"/>
-        <v>126</v>
-      </c>
-      <c r="B128">
-        <f t="shared" ref="B128" si="120">B126+1</f>
-        <v>63</v>
-      </c>
-      <c r="C128" t="s">
-        <v>239</v>
-      </c>
-      <c r="D128" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A129">
-        <f t="shared" si="61"/>
-        <v>127</v>
-      </c>
-      <c r="B129">
-        <f t="shared" ref="B129" si="121">B128</f>
-        <v>63</v>
-      </c>
-      <c r="C129" t="s">
-        <v>238</v>
-      </c>
-      <c r="D129" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A130">
-        <f t="shared" si="61"/>
-        <v>128</v>
-      </c>
-      <c r="B130">
-        <f t="shared" ref="B130" si="122">B128+1</f>
-        <v>64</v>
-      </c>
-      <c r="C130" t="s">
-        <v>237</v>
-      </c>
-      <c r="D130" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A131">
-        <f t="shared" si="61"/>
-        <v>129</v>
-      </c>
-      <c r="B131">
-        <f t="shared" ref="B131" si="123">B130</f>
-        <v>64</v>
-      </c>
-      <c r="C131" t="s">
-        <v>236</v>
-      </c>
-      <c r="D131" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A132">
-        <f t="shared" si="61"/>
-        <v>130</v>
-      </c>
-      <c r="B132">
-        <f t="shared" ref="B132" si="124">B130+1</f>
-        <v>65</v>
-      </c>
-      <c r="C132" t="s">
-        <v>235</v>
-      </c>
-      <c r="D132" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A133">
-        <f t="shared" si="61"/>
-        <v>131</v>
-      </c>
-      <c r="B133">
-        <f t="shared" ref="B133" si="125">B132</f>
-        <v>65</v>
-      </c>
-      <c r="C133" t="s">
-        <v>234</v>
-      </c>
-      <c r="D133" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A134">
-        <f t="shared" ref="A134:A139" si="126">A133+1</f>
-        <v>132</v>
-      </c>
-      <c r="B134">
-        <f t="shared" ref="B134" si="127">B132+1</f>
-        <v>66</v>
-      </c>
-      <c r="C134" t="s">
-        <v>233</v>
-      </c>
-      <c r="D134" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A135">
-        <f t="shared" si="126"/>
-        <v>133</v>
-      </c>
-      <c r="B135">
-        <f t="shared" ref="B135" si="128">B134</f>
-        <v>66</v>
-      </c>
-      <c r="C135" t="s">
-        <v>232</v>
-      </c>
-      <c r="D135" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A136">
-        <f t="shared" si="126"/>
-        <v>134</v>
-      </c>
-      <c r="B136">
-        <f>B134+1</f>
-        <v>67</v>
-      </c>
-      <c r="C136" t="s">
-        <v>231</v>
-      </c>
-      <c r="D136" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A137">
-        <f t="shared" si="126"/>
-        <v>135</v>
-      </c>
-      <c r="B137">
-        <f t="shared" ref="B137:B139" si="129">B136</f>
-        <v>67</v>
-      </c>
-      <c r="C137" t="s">
-        <v>230</v>
-      </c>
-      <c r="D137" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A138">
-        <f t="shared" si="126"/>
-        <v>136</v>
-      </c>
-      <c r="B138">
-        <f>B137+1</f>
-        <v>68</v>
-      </c>
-      <c r="C138" t="s">
-        <v>229</v>
-      </c>
-      <c r="D138" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A139">
-        <f t="shared" si="126"/>
-        <v>137</v>
-      </c>
-      <c r="B139">
-        <f t="shared" si="129"/>
-        <v>68</v>
-      </c>
-      <c r="C139" t="s">
-        <v>228</v>
-      </c>
-      <c r="D139" t="s">
         <v>204</v>
       </c>
     </row>

</xml_diff>

<commit_message>
clean up, saturate coh sum instead of samples
</commit_message>
<xml_diff>
--- a/doc/flower-register-map.xlsx
+++ b/doc/flower-register-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\dev\FLOWER-board-firmware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69701C28-00A0-4286-996E-2D1F345790AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642C969E-A069-487E-936E-D89E77AE0FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registers" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="255">
   <si>
     <t>Register Map</t>
   </si>
@@ -778,6 +778,30 @@
   </si>
   <si>
     <t>lower 12 bits are threshold offset (ie. Bumps all SBC thresholds up by x amount)</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 1 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 2 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 3 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 4 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 5 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 6 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 7 thresholds</t>
+  </si>
+  <si>
+    <t>phased trigger-&gt; beam 8 thresholds</t>
   </si>
 </sst>
 </file>
@@ -979,7 +1003,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1076,6 +1100,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3587,7 +3612,7 @@
         <v>x81</v>
       </c>
       <c r="C136" s="40" t="s">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="D136" s="40" t="s">
         <v>228</v>
@@ -3606,7 +3631,7 @@
         <v>x82</v>
       </c>
       <c r="C137" s="40" t="s">
-        <v>227</v>
+        <v>248</v>
       </c>
       <c r="D137" s="40" t="s">
         <v>228</v>
@@ -3625,7 +3650,7 @@
         <v>x83</v>
       </c>
       <c r="C138" s="40" t="s">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="D138" s="40" t="s">
         <v>228</v>
@@ -3644,7 +3669,7 @@
         <v>x84</v>
       </c>
       <c r="C139" s="40" t="s">
-        <v>227</v>
+        <v>250</v>
       </c>
       <c r="D139" s="40" t="s">
         <v>228</v>
@@ -3663,7 +3688,7 @@
         <v>x85</v>
       </c>
       <c r="C140" s="40" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
       <c r="D140" s="40" t="s">
         <v>228</v>
@@ -3682,7 +3707,7 @@
         <v>x86</v>
       </c>
       <c r="C141" s="40" t="s">
-        <v>227</v>
+        <v>252</v>
       </c>
       <c r="D141" s="40" t="s">
         <v>228</v>
@@ -3701,7 +3726,7 @@
         <v>x87</v>
       </c>
       <c r="C142" s="40" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="D142" s="40" t="s">
         <v>228</v>
@@ -3720,7 +3745,7 @@
         <v>x88</v>
       </c>
       <c r="C143" s="40" t="s">
-        <v>227</v>
+        <v>254</v>
       </c>
       <c r="D143" s="40" t="s">
         <v>228</v>
@@ -3738,15 +3763,9 @@
         <f t="shared" si="5"/>
         <v>x89</v>
       </c>
-      <c r="C144" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D144" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E144" s="40" t="s">
-        <v>229</v>
-      </c>
+      <c r="C144" s="46"/>
+      <c r="D144" s="46"/>
+      <c r="E144" s="46"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145">
@@ -3757,15 +3776,9 @@
         <f t="shared" si="5"/>
         <v>x8A</v>
       </c>
-      <c r="C145" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D145" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E145" s="40" t="s">
-        <v>229</v>
-      </c>
+      <c r="C145" s="46"/>
+      <c r="D145" s="46"/>
+      <c r="E145" s="46"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146">
@@ -3776,15 +3789,9 @@
         <f t="shared" si="5"/>
         <v>x8B</v>
       </c>
-      <c r="C146" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D146" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E146" s="40" t="s">
-        <v>229</v>
-      </c>
+      <c r="C146" s="46"/>
+      <c r="D146" s="46"/>
+      <c r="E146" s="46"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147">
@@ -3795,15 +3802,6 @@
         <f t="shared" si="5"/>
         <v>x8C</v>
       </c>
-      <c r="C147" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D147" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E147" s="40" t="s">
-        <v>229</v>
-      </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
@@ -3814,15 +3812,6 @@
         <f t="shared" si="5"/>
         <v>x8D</v>
       </c>
-      <c r="C148" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D148" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E148" s="40" t="s">
-        <v>229</v>
-      </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149">
@@ -3833,15 +3822,6 @@
         <f t="shared" si="5"/>
         <v>x8E</v>
       </c>
-      <c r="C149" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D149" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E149" s="40" t="s">
-        <v>229</v>
-      </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150">
@@ -3851,15 +3831,6 @@
       <c r="B150" s="16" t="str">
         <f t="shared" si="5"/>
         <v>x8F</v>
-      </c>
-      <c r="C150" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D150" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="E150" s="40" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
@@ -6092,7 +6063,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70">
-        <f t="shared" ref="A70:A133" si="61">A69+1</f>
+        <f t="shared" ref="A70:A97" si="61">A69+1</f>
         <v>68</v>
       </c>
       <c r="B70">

</xml_diff>

<commit_message>
refactor some things, lower power trigger step to 1 real sample, correct triggering channels to data manager
</commit_message>
<xml_diff>
--- a/doc/flower-register-map.xlsx
+++ b/doc/flower-register-map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\dev\FLOWER-board-firmware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{015CDA2A-6F70-4FDF-9EEE-55169E325FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A504BD9E-65F3-49C9-BE3B-D66890D3703F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="261">
   <si>
     <t>Register Map</t>
   </si>
@@ -814,6 +814,12 @@
   </si>
   <si>
     <t>high byte contains station that the firmware was compile for</t>
+  </si>
+  <si>
+    <t>READ ONLY</t>
+  </si>
+  <si>
+    <t>test burst read</t>
   </si>
 </sst>
 </file>
@@ -929,7 +935,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1017,11 +1023,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1118,7 +1133,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1492,8 +1515,11 @@
         <v>66</v>
       </c>
       <c r="F7"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G7" s="46" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1507,6 +1533,7 @@
       <c r="D8" t="s">
         <v>16</v>
       </c>
+      <c r="G8" s="47"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -1526,6 +1553,7 @@
       <c r="F9" s="3" t="s">
         <v>258</v>
       </c>
+      <c r="G9" s="47"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
@@ -1545,6 +1573,7 @@
       <c r="F10" s="3" t="s">
         <v>80</v>
       </c>
+      <c r="G10" s="47"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
@@ -1564,6 +1593,7 @@
       <c r="F11" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="G11" s="47"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
@@ -1583,6 +1613,7 @@
       <c r="F12" s="3" t="s">
         <v>28</v>
       </c>
+      <c r="G12" s="47"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
@@ -1602,6 +1633,7 @@
       <c r="F13" s="3" t="s">
         <v>85</v>
       </c>
+      <c r="G13" s="47"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
@@ -1618,6 +1650,7 @@
       <c r="D14" t="s">
         <v>159</v>
       </c>
+      <c r="G14" s="47"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -1634,6 +1667,7 @@
       <c r="D15" s="34" t="s">
         <v>16</v>
       </c>
+      <c r="G15" s="47"/>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16">
@@ -1650,8 +1684,9 @@
       <c r="D16" s="34" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" s="47"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <f t="shared" si="1"/>
         <v>10</v>
@@ -1672,8 +1707,9 @@
       <c r="F17" s="11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" s="47"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="12">
         <f t="shared" si="1"/>
         <v>11</v>
@@ -1692,8 +1728,9 @@
         <v>6</v>
       </c>
       <c r="F18" s="13"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" s="47"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="12">
         <f t="shared" si="1"/>
         <v>12</v>
@@ -1712,8 +1749,9 @@
         <v>6</v>
       </c>
       <c r="F19" s="13"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" s="47"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="12">
         <f t="shared" si="1"/>
         <v>13</v>
@@ -1732,8 +1770,9 @@
         <v>6</v>
       </c>
       <c r="F20" s="13"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" s="47"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="12">
         <f t="shared" si="1"/>
         <v>14</v>
@@ -1752,8 +1791,9 @@
         <v>6</v>
       </c>
       <c r="F21" s="13"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21" s="47"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="12">
         <f t="shared" si="1"/>
         <v>15</v>
@@ -1769,8 +1809,9 @@
         <v>168</v>
       </c>
       <c r="F22" s="13"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22" s="47"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="12">
         <f t="shared" si="1"/>
         <v>16</v>
@@ -1789,8 +1830,9 @@
         <v>6</v>
       </c>
       <c r="F23" s="13"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23" s="47"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="12">
         <f t="shared" si="1"/>
         <v>17</v>
@@ -1809,8 +1851,9 @@
         <v>6</v>
       </c>
       <c r="F24" s="13"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G24" s="47"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="12">
         <f t="shared" si="1"/>
         <v>18</v>
@@ -1829,8 +1872,9 @@
         <v>6</v>
       </c>
       <c r="F25" s="13"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25" s="47"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="12">
         <f t="shared" si="1"/>
         <v>19</v>
@@ -1840,8 +1884,9 @@
         <v>x13</v>
       </c>
       <c r="F26" s="13"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26" s="47"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="12">
         <f t="shared" si="1"/>
         <v>20</v>
@@ -1851,8 +1896,9 @@
         <v>x14</v>
       </c>
       <c r="F27" s="13"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27" s="47"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="12">
         <f t="shared" si="1"/>
         <v>21</v>
@@ -1862,8 +1908,9 @@
         <v>x15</v>
       </c>
       <c r="F28" s="13"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" s="47"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="12">
         <f t="shared" si="1"/>
         <v>22</v>
@@ -1873,8 +1920,9 @@
         <v>x16</v>
       </c>
       <c r="F29" s="13"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" s="47"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="12">
         <f t="shared" si="1"/>
         <v>23</v>
@@ -1884,8 +1932,9 @@
         <v>x17</v>
       </c>
       <c r="F30" s="13"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" s="47"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="12">
         <f t="shared" si="1"/>
         <v>24</v>
@@ -1895,8 +1944,9 @@
         <v>x18</v>
       </c>
       <c r="F31" s="13"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31" s="47"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="12">
         <f t="shared" si="1"/>
         <v>25</v>
@@ -1906,8 +1956,9 @@
         <v>x19</v>
       </c>
       <c r="F32" s="13"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32" s="47"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12">
         <f t="shared" si="1"/>
         <v>26</v>
@@ -1917,8 +1968,9 @@
         <v>x1A</v>
       </c>
       <c r="F33" s="13"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33" s="47"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="12">
         <f t="shared" si="1"/>
         <v>27</v>
@@ -1928,8 +1980,9 @@
         <v>x1B</v>
       </c>
       <c r="F34" s="13"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34" s="47"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="12">
         <f t="shared" si="1"/>
         <v>28</v>
@@ -1939,8 +1992,9 @@
         <v>x1C</v>
       </c>
       <c r="F35" s="13"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35" s="47"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="12">
         <f t="shared" si="1"/>
         <v>29</v>
@@ -1950,8 +2004,9 @@
         <v>x1D</v>
       </c>
       <c r="F36" s="13"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G36" s="47"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="12">
         <f t="shared" si="1"/>
         <v>30</v>
@@ -1961,8 +2016,9 @@
         <v>x1E</v>
       </c>
       <c r="F37" s="13"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37" s="47"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="12">
         <f t="shared" si="1"/>
         <v>31</v>
@@ -1972,8 +2028,9 @@
         <v>x1F</v>
       </c>
       <c r="F38" s="13"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" s="47"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="12">
         <f t="shared" si="1"/>
         <v>32</v>
@@ -1983,8 +2040,9 @@
         <v>x20</v>
       </c>
       <c r="F39" s="13"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" s="47"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="12">
         <f t="shared" si="1"/>
         <v>33</v>
@@ -1994,8 +2052,9 @@
         <v>x21</v>
       </c>
       <c r="F40" s="13"/>
-    </row>
-    <row r="41" spans="1:6" s="25" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G40" s="47"/>
+    </row>
+    <row r="41" spans="1:7" s="25" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="28">
         <f t="shared" si="1"/>
         <v>34</v>
@@ -2010,8 +2069,9 @@
       <c r="D41" s="30"/>
       <c r="E41" s="30"/>
       <c r="F41" s="31"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" s="48"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <f t="shared" si="1"/>
         <v>35</v>
@@ -2030,7 +2090,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <f t="shared" si="1"/>
         <v>36</v>
@@ -2049,7 +2109,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <f t="shared" si="1"/>
         <v>37</v>
@@ -2068,7 +2128,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <f t="shared" si="1"/>
         <v>38</v>
@@ -2087,7 +2147,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="37">
         <f t="shared" si="1"/>
         <v>39</v>
@@ -2109,7 +2169,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <f t="shared" si="1"/>
         <v>40</v>
@@ -2128,7 +2188,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <f t="shared" si="1"/>
         <v>41</v>
@@ -2239,6 +2299,9 @@
         <f t="shared" si="0"/>
         <v>x2F</v>
       </c>
+      <c r="C54" t="s">
+        <v>260</v>
+      </c>
       <c r="D54" s="3"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -3841,8 +3904,6 @@
         <f t="shared" si="5"/>
         <v>x8C</v>
       </c>
-      <c r="C147" s="46"/>
-      <c r="D147" s="46"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
@@ -3853,8 +3914,6 @@
         <f t="shared" si="5"/>
         <v>x8D</v>
       </c>
-      <c r="C148" s="46"/>
-      <c r="D148" s="46"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149">
@@ -3865,8 +3924,6 @@
         <f t="shared" si="5"/>
         <v>x8E</v>
       </c>
-      <c r="C149" s="46"/>
-      <c r="D149" s="46"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150">
@@ -3877,8 +3934,6 @@
         <f t="shared" si="5"/>
         <v>x8F</v>
       </c>
-      <c r="C150" s="46"/>
-      <c r="D150" s="46"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151">
@@ -5001,11 +5056,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G7:G41"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fine gain equalization, fix bad rounding code
</commit_message>
<xml_diff>
--- a/doc/flower-register-map.xlsx
+++ b/doc/flower-register-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\dev\FLOWER-board-firmware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A504BD9E-65F3-49C9-BE3B-D66890D3703F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FEC9C1-0186-4825-89E4-A8335B3258A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registers" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="265">
   <si>
     <t>Register Map</t>
   </si>
@@ -820,6 +820,18 @@
   </si>
   <si>
     <t>test burst read</t>
+  </si>
+  <si>
+    <t>phased trigger -&gt; ch0 and ch1 fine gain equalization</t>
+  </si>
+  <si>
+    <t>phased trigger -&gt; ch2 and ch3 fine gain equalization</t>
+  </si>
+  <si>
+    <t>First byte, lower 5 bits for ch 0. Second byte, lower 5 bits for ch 1. (64-number)*samples/64</t>
+  </si>
+  <si>
+    <t>First byte, lower 5 bits for ch 2. Second byte, lower 5 bits for ch 3. (64-number)*samples/64</t>
   </si>
 </sst>
 </file>
@@ -1136,7 +1148,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3904,6 +3916,15 @@
         <f t="shared" si="5"/>
         <v>x8C</v>
       </c>
+      <c r="C147" s="40" t="s">
+        <v>261</v>
+      </c>
+      <c r="D147" s="40" t="s">
+        <v>263</v>
+      </c>
+      <c r="E147" s="40" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
@@ -3913,6 +3934,15 @@
       <c r="B148" s="16" t="str">
         <f t="shared" si="5"/>
         <v>x8D</v>
+      </c>
+      <c r="C148" s="40" t="s">
+        <v>262</v>
+      </c>
+      <c r="D148" s="40" t="s">
+        <v>264</v>
+      </c>
+      <c r="E148" s="40" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Revert "fine gain equalization, fix bad rounding code"
This reverts commit 65b2a26a64ae7f30957e0b4655d36ecdd1dd6262.
</commit_message>
<xml_diff>
--- a/doc/flower-register-map.xlsx
+++ b/doc/flower-register-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\dev\FLOWER-board-firmware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FEC9C1-0186-4825-89E4-A8335B3258A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A504BD9E-65F3-49C9-BE3B-D66890D3703F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registers" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="261">
   <si>
     <t>Register Map</t>
   </si>
@@ -820,18 +820,6 @@
   </si>
   <si>
     <t>test burst read</t>
-  </si>
-  <si>
-    <t>phased trigger -&gt; ch0 and ch1 fine gain equalization</t>
-  </si>
-  <si>
-    <t>phased trigger -&gt; ch2 and ch3 fine gain equalization</t>
-  </si>
-  <si>
-    <t>First byte, lower 5 bits for ch 0. Second byte, lower 5 bits for ch 1. (64-number)*samples/64</t>
-  </si>
-  <si>
-    <t>First byte, lower 5 bits for ch 2. Second byte, lower 5 bits for ch 3. (64-number)*samples/64</t>
   </si>
 </sst>
 </file>
@@ -1148,7 +1136,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3916,15 +3904,6 @@
         <f t="shared" si="5"/>
         <v>x8C</v>
       </c>
-      <c r="C147" s="40" t="s">
-        <v>261</v>
-      </c>
-      <c r="D147" s="40" t="s">
-        <v>263</v>
-      </c>
-      <c r="E147" s="40" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
@@ -3934,15 +3913,6 @@
       <c r="B148" s="16" t="str">
         <f t="shared" si="5"/>
         <v>x8D</v>
-      </c>
-      <c r="C148" s="40" t="s">
-        <v>262</v>
-      </c>
-      <c r="D148" s="40" t="s">
-        <v>264</v>
-      </c>
-      <c r="E148" s="40" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
document beam delays and update reg file
</commit_message>
<xml_diff>
--- a/doc/flower-register-map.xlsx
+++ b/doc/flower-register-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryank\Documents\firmware\rnog\dev\FLOWER-board-firmware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A504BD9E-65F3-49C9-BE3B-D66890D3703F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85451262-C064-4DD7-9442-C5949AFC11AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="228" windowWidth="17280" windowHeight="8964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registers" sheetId="1" r:id="rId1"/>
@@ -1136,7 +1136,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">

</xml_diff>